<commit_message>
Updating activity log copy
</commit_message>
<xml_diff>
--- a/supporting documents/Project Activity Log.xlsx
+++ b/supporting documents/Project Activity Log.xlsx
@@ -15,14 +15,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId11" roundtripDataChecksum="CZefYtqh5YhrUMUmA6V9hnYvXijTYjSlqKS1oD3+0GE="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId11" roundtripDataChecksum="gMYxjJ0S1AQ8bS3GC1M6VjQrIYrvmcr4pzFz5HrLu/M="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="915" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="959" uniqueCount="304">
   <si>
     <t>Name:</t>
   </si>
@@ -116,6 +116,12 @@
     <t>5mins</t>
   </si>
   <si>
+    <t>Completed written proposal document and added it to the drive</t>
+  </si>
+  <si>
+    <t>1hr</t>
+  </si>
+  <si>
     <t>Attended group meeting to discuss preliminary draft of Question 1 - 4 of  CFG Data Project Question Guide</t>
   </si>
   <si>
@@ -128,7 +134,58 @@
     <t>Suggested delegation of tasks but this should take shape once project is finally approved by instructor</t>
   </si>
   <si>
-    <t xml:space="preserve">Suggested familiarity with primary dataset before the next meeting to minimize </t>
+    <t>Suggested familiarity with primary dataset before the next meeting to minimize delay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attended group call to discuss roles and responsibilities, task focused on data cleaning </t>
+  </si>
+  <si>
+    <t>30 mins</t>
+  </si>
+  <si>
+    <t>Group call to discuss work progress</t>
+  </si>
+  <si>
+    <t>30mins</t>
+  </si>
+  <si>
+    <t>Started Data cleaning and shared Data Cleaning with May for dataset assigned to May &amp; I(May Suggested ti use her Cleaned Data for our group)</t>
+  </si>
+  <si>
+    <t>1 hr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attended Group Meeting </t>
+  </si>
+  <si>
+    <t>Attended Group Call</t>
+  </si>
+  <si>
+    <t>50 mins</t>
+  </si>
+  <si>
+    <t>Completed Readme for the cleaning notebook</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1hr </t>
+  </si>
+  <si>
+    <t>Completed Summary Key Finding Documentation</t>
+  </si>
+  <si>
+    <t>35mins</t>
+  </si>
+  <si>
+    <t>Refined Data set to get a different analysis - Correlation Matrix</t>
+  </si>
+  <si>
+    <t>2hours</t>
+  </si>
+  <si>
+    <t>Created a slide for presentation</t>
+  </si>
+  <si>
+    <t>15mins</t>
   </si>
   <si>
     <r>
@@ -183,18 +240,12 @@
     <t>Researched datasets and started working on ideas for project</t>
   </si>
   <si>
-    <t>1 hr</t>
-  </si>
-  <si>
     <t>14/11/2025</t>
   </si>
   <si>
     <t>Team call to discuss initial ideas and next steps, agreed to work on odeas over weekend and discuss on Monday</t>
   </si>
   <si>
-    <t>30 mins</t>
-  </si>
-  <si>
     <t>17/11/2025</t>
   </si>
   <si>
@@ -220,9 +271,6 @@
   </si>
   <si>
     <t>Group call to discuss proposal document</t>
-  </si>
-  <si>
-    <t>50 mins</t>
   </si>
   <si>
     <t>20/11/2025</t>
@@ -1201,6 +1249,9 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -1209,9 +1260,6 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
@@ -1707,16 +1755,16 @@
         <v>2.0</v>
       </c>
       <c r="B13" s="9">
-        <v>45980.0</v>
+        <v>45978.0</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>26</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>13</v>
@@ -1731,13 +1779,13 @@
         <v>45980.0</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>13</v>
@@ -1755,13 +1803,13 @@
         <v>29</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>19</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G15" s="3"/>
     </row>
@@ -1773,7 +1821,7 @@
         <v>45980.0</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>18</v>
@@ -1782,107 +1830,239 @@
         <v>19</v>
       </c>
       <c r="F16" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="3"/>
+    </row>
+    <row r="17" ht="15.75" customHeight="1">
+      <c r="A17" s="8">
+        <v>2.0</v>
+      </c>
+      <c r="B17" s="9">
+        <v>45980.0</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="G16" s="3"/>
-    </row>
-    <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
+      <c r="E17" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="G17" s="3"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
+      <c r="A18" s="8">
+        <v>3.0</v>
+      </c>
+      <c r="B18" s="9">
+        <v>45985.0</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="G18" s="3"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
+      <c r="A19" s="8">
+        <v>3.0</v>
+      </c>
+      <c r="B19" s="10">
+        <v>45988.0</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="G19" s="3"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
+      <c r="A20" s="8">
+        <v>4.0</v>
+      </c>
+      <c r="B20" s="10">
+        <v>45994.0</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="G20" s="3"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
+      <c r="A21" s="8">
+        <v>4.0</v>
+      </c>
+      <c r="B21" s="10">
+        <v>45996.0</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="G21" s="3"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
+      <c r="A22" s="8">
+        <v>5.0</v>
+      </c>
+      <c r="B22" s="10">
+        <v>45999.0</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="G22" s="3"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
+      <c r="A23" s="8">
+        <v>5.0</v>
+      </c>
+      <c r="B23" s="9">
+        <v>46001.0</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="G23" s="3"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
+      <c r="A24" s="8">
+        <v>5.0</v>
+      </c>
+      <c r="B24" s="9">
+        <v>46002.0</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="G24" s="3"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
+      <c r="A25" s="8">
+        <v>5.0</v>
+      </c>
+      <c r="B25" s="9">
+        <v>46003.0</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="G25" s="3"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
+      <c r="A26" s="8">
+        <v>5.0</v>
+      </c>
+      <c r="B26" s="9">
+        <v>46004.0</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="G26" s="3"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
+      <c r="A27" s="8">
+        <v>5.0</v>
+      </c>
+      <c r="B27" s="9">
+        <v>46004.0</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="G27" s="3"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
@@ -2078,17 +2258,49 @@
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
-      <c r="D49" s="3" t="s">
-        <v>31</v>
-      </c>
+      <c r="D49" s="3"/>
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1"/>
-    <row r="51" ht="15.75" customHeight="1"/>
-    <row r="52" ht="15.75" customHeight="1"/>
-    <row r="53" ht="15.75" customHeight="1"/>
+    <row r="50" ht="15.75" customHeight="1">
+      <c r="A50" s="3"/>
+      <c r="B50" s="3"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+    </row>
+    <row r="51" ht="15.75" customHeight="1">
+      <c r="A51" s="3"/>
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+    </row>
+    <row r="52" ht="15.75" customHeight="1">
+      <c r="A52" s="3"/>
+      <c r="B52" s="3"/>
+      <c r="C52" s="3"/>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+    </row>
+    <row r="53" ht="15.75" customHeight="1">
+      <c r="A53" s="3"/>
+      <c r="B53" s="3"/>
+      <c r="C53" s="3"/>
+      <c r="D53" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E53" s="3"/>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3"/>
+    </row>
     <row r="54" ht="15.75" customHeight="1"/>
     <row r="55" ht="15.75" customHeight="1"/>
     <row r="56" ht="15.75" customHeight="1"/>
@@ -3036,6 +3248,10 @@
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
+    <row r="1001" ht="15.75" customHeight="1"/>
+    <row r="1002" ht="15.75" customHeight="1"/>
+    <row r="1003" ht="15.75" customHeight="1"/>
+    <row r="1004" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:G1"/>
@@ -3069,10 +3285,10 @@
         <v>0</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>33</v>
+        <v>51</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>52</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
@@ -3080,7 +3296,7 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" ht="29.25" customHeight="1"/>
@@ -3120,8 +3336,8 @@
       <c r="A7" s="6">
         <v>1.0</v>
       </c>
-      <c r="B7" s="11" t="s">
-        <v>35</v>
+      <c r="B7" s="12" t="s">
+        <v>54</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>10</v>
@@ -3143,17 +3359,17 @@
       <c r="A8" s="8">
         <v>1.0</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="13">
         <v>46002.0</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>13</v>
@@ -3165,16 +3381,16 @@
         <v>1.0</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="C9" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="8" t="s">
-        <v>39</v>
-      </c>
       <c r="E9" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>13</v>
@@ -3186,13 +3402,13 @@
         <v>1.0</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>16</v>
@@ -3207,16 +3423,16 @@
         <v>2.0</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>13</v>
@@ -3228,16 +3444,16 @@
         <v>2.0</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>13</v>
@@ -3249,10 +3465,10 @@
         <v>2.0</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>23</v>
@@ -3270,16 +3486,16 @@
         <v>2.0</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>13</v>
@@ -3291,16 +3507,16 @@
         <v>2.0</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>23</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>13</v>
@@ -3312,13 +3528,13 @@
         <v>2.0</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E16" s="8" t="s">
         <v>16</v>
@@ -3333,16 +3549,16 @@
         <v>2.0</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F17" s="8" t="s">
         <v>13</v>
@@ -3354,13 +3570,13 @@
         <v>3.0</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E18" s="8" t="s">
         <v>16</v>
@@ -3369,7 +3585,7 @@
         <v>13</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19">
@@ -3377,16 +3593,16 @@
         <v>3.0</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>13</v>
@@ -3398,16 +3614,16 @@
         <v>3.0</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>13</v>
@@ -3419,16 +3635,16 @@
         <v>3.0</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F21" s="8" t="s">
         <v>13</v>
@@ -3440,13 +3656,13 @@
         <v>3.0</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="E22" s="8" t="s">
         <v>16</v>
@@ -3461,16 +3677,16 @@
         <v>3.0</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="D23" s="8" t="s">
         <v>23</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F23" s="8" t="s">
         <v>13</v>
@@ -3481,17 +3697,17 @@
       <c r="A24" s="8">
         <v>4.0</v>
       </c>
-      <c r="B24" s="13">
+      <c r="B24" s="10">
         <v>45669.0</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F24" s="8" t="s">
         <v>13</v>
@@ -3502,17 +3718,17 @@
       <c r="A25" s="8">
         <v>4.0</v>
       </c>
-      <c r="B25" s="13">
+      <c r="B25" s="10">
         <v>45669.0</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F25" s="8" t="s">
         <v>13</v>
@@ -3523,14 +3739,14 @@
       <c r="A26" s="8">
         <v>4.0</v>
       </c>
-      <c r="B26" s="13">
+      <c r="B26" s="10">
         <v>45669.0</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E26" s="8" t="s">
         <v>16</v>
@@ -3539,24 +3755,24 @@
         <v>13</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="8">
         <v>4.0</v>
       </c>
-      <c r="B27" s="13">
+      <c r="B27" s="10">
         <v>45700.0</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>74</v>
+        <v>90</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F27" s="8" t="s">
         <v>13</v>
@@ -3567,17 +3783,17 @@
       <c r="A28" s="8">
         <v>4.0</v>
       </c>
-      <c r="B28" s="13">
+      <c r="B28" s="10">
         <v>45700.0</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F28" s="8" t="s">
         <v>13</v>
@@ -3588,17 +3804,17 @@
       <c r="A29" s="8">
         <v>4.0</v>
       </c>
-      <c r="B29" s="13">
+      <c r="B29" s="10">
         <v>45728.0</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F29" s="8" t="s">
         <v>13</v>
@@ -3609,17 +3825,17 @@
       <c r="A30" s="8">
         <v>4.0</v>
       </c>
-      <c r="B30" s="13">
+      <c r="B30" s="10">
         <v>45728.0</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F30" s="8" t="s">
         <v>13</v>
@@ -3630,14 +3846,14 @@
       <c r="A31" s="8">
         <v>4.0</v>
       </c>
-      <c r="B31" s="13">
+      <c r="B31" s="10">
         <v>45728.0</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="E31" s="8" t="s">
         <v>16</v>
@@ -3651,17 +3867,17 @@
       <c r="A32" s="8">
         <v>4.0</v>
       </c>
-      <c r="B32" s="13">
+      <c r="B32" s="10">
         <v>45759.0</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F32" s="8" t="s">
         <v>13</v>
@@ -3672,17 +3888,17 @@
       <c r="A33" s="8">
         <v>4.0</v>
       </c>
-      <c r="B33" s="13">
+      <c r="B33" s="10">
         <v>45759.0</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F33" s="8" t="s">
         <v>13</v>
@@ -3693,17 +3909,17 @@
       <c r="A34" s="8">
         <v>4.0</v>
       </c>
-      <c r="B34" s="13">
+      <c r="B34" s="10">
         <v>45759.0</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F34" s="8" t="s">
         <v>13</v>
@@ -3714,17 +3930,17 @@
       <c r="A35" s="8">
         <v>4.0</v>
       </c>
-      <c r="B35" s="13">
+      <c r="B35" s="10">
         <v>45789.0</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="D35" s="8" t="s">
         <v>23</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F35" s="8" t="s">
         <v>13</v>
@@ -3735,17 +3951,17 @@
       <c r="A36" s="8">
         <v>4.0</v>
       </c>
-      <c r="B36" s="13">
+      <c r="B36" s="10">
         <v>45789.0</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F36" s="8" t="s">
         <v>13</v>
@@ -3756,17 +3972,17 @@
       <c r="A37" s="8">
         <v>4.0</v>
       </c>
-      <c r="B37" s="13">
+      <c r="B37" s="10">
         <v>45820.0</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F37" s="8" t="s">
         <v>13</v>
@@ -3777,17 +3993,17 @@
       <c r="A38" s="8">
         <v>5.0</v>
       </c>
-      <c r="B38" s="13">
+      <c r="B38" s="10">
         <v>45881.0</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F38" s="8" t="s">
         <v>13</v>
@@ -3798,17 +4014,17 @@
       <c r="A39" s="8">
         <v>5.0</v>
       </c>
-      <c r="B39" s="13">
+      <c r="B39" s="10">
         <v>45881.0</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F39" s="8" t="s">
         <v>13</v>
@@ -3819,17 +4035,17 @@
       <c r="A40" s="8">
         <v>5.0</v>
       </c>
-      <c r="B40" s="13">
+      <c r="B40" s="10">
         <v>45912.0</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="D40" s="8" t="s">
         <v>23</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F40" s="8" t="s">
         <v>13</v>
@@ -3844,7 +4060,7 @@
         <v>45942.0</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="D41" s="8" t="s">
         <v>23</v>
@@ -3865,13 +4081,13 @@
         <v>45973.0</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F42" s="8" t="s">
         <v>13</v>
@@ -3886,13 +4102,13 @@
         <v>46003.0</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F43" s="8" t="s">
         <v>13</v>
@@ -3985,7 +4201,7 @@
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
       <c r="D53" s="3" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
@@ -6877,10 +7093,10 @@
         <v>0</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>33</v>
+        <v>111</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>52</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
@@ -6888,7 +7104,7 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>96</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" ht="29.25" customHeight="1"/>
@@ -6915,7 +7131,7 @@
         <v>6</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>8</v>
@@ -6928,17 +7144,17 @@
       <c r="A7" s="8">
         <v>1.0</v>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="13">
         <v>45941.0</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F7" s="8" t="s">
         <v>13</v>
@@ -6950,22 +7166,22 @@
         <v>1.0</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9">
@@ -6973,22 +7189,22 @@
         <v>1.0</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -6996,22 +7212,22 @@
         <v>2.0</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -7019,22 +7235,22 @@
         <v>2.0</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -7042,16 +7258,16 @@
         <v>2.0</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="C12" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="E12" s="8" t="s">
         <v>111</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>95</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>13</v>
@@ -7063,16 +7279,16 @@
         <v>2.0</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>13</v>
@@ -7084,16 +7300,16 @@
         <v>3.0</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>13</v>
@@ -7105,22 +7321,22 @@
         <v>3.0</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>114</v>
+        <v>130</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
@@ -7131,19 +7347,19 @@
         <v>45669.0</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>116</v>
+        <v>132</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>117</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
@@ -7154,13 +7370,13 @@
         <v>45669.0</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="D17" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F17" s="8" t="s">
         <v>13</v>
@@ -7175,13 +7391,13 @@
         <v>45728.0</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>13</v>
@@ -7196,13 +7412,13 @@
         <v>45728.0</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>13</v>
@@ -7217,13 +7433,13 @@
         <v>45789.0</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>13</v>
@@ -7238,13 +7454,13 @@
         <v>45789.0</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>120</v>
+        <v>136</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="F21" s="8" t="s">
         <v>13</v>
@@ -7259,13 +7475,13 @@
         <v>45789.0</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F22" s="8" t="s">
         <v>13</v>
@@ -7280,13 +7496,13 @@
         <v>45881.0</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F23" s="8" t="s">
         <v>13</v>
@@ -7301,13 +7517,13 @@
         <v>45912.0</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>121</v>
+        <v>137</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>122</v>
+        <v>138</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="F24" s="8" t="s">
         <v>13</v>
@@ -7322,13 +7538,13 @@
         <v>45942.0</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F25" s="8" t="s">
         <v>13</v>
@@ -7343,13 +7559,13 @@
         <v>45973.0</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="F26" s="8" t="s">
         <v>13</v>
@@ -7364,13 +7580,13 @@
         <v>46003.0</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F27" s="8" t="s">
         <v>13</v>
@@ -7382,17 +7598,17 @@
         <v>6.0</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="D28" s="8"/>
       <c r="E28" s="8" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>126</v>
+        <v>142</v>
       </c>
       <c r="G28" s="3"/>
     </row>
@@ -7427,7 +7643,7 @@
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="18" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
@@ -7601,7 +7817,7 @@
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
       <c r="D51" s="3" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
@@ -8595,12 +8811,12 @@
       <c r="A1" s="1"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="10" t="s">
-        <v>129</v>
+      <c r="A2" s="11" t="s">
+        <v>145</v>
       </c>
       <c r="B2" s="3"/>
-      <c r="C2" s="10" t="s">
-        <v>130</v>
+      <c r="C2" s="11" t="s">
+        <v>146</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
@@ -8608,7 +8824,7 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4" ht="29.25" customHeight="1"/>
@@ -8645,22 +8861,22 @@
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="11">
+      <c r="A7" s="12">
         <v>1.0</v>
       </c>
-      <c r="B7" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="F7" s="11" t="s">
+      <c r="B7" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="F7" s="12" t="s">
         <v>13</v>
       </c>
       <c r="G7" s="6"/>
@@ -8669,17 +8885,17 @@
       <c r="A8" s="6">
         <v>1.0</v>
       </c>
-      <c r="B8" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>134</v>
+      <c r="B8" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>150</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>13</v>
@@ -8691,19 +8907,19 @@
         <v>1.0</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>136</v>
+        <v>152</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>137</v>
+        <v>153</v>
       </c>
       <c r="G9" s="3"/>
     </row>
@@ -8712,16 +8928,16 @@
         <v>1.0</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>138</v>
+        <v>154</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>13</v>
@@ -8733,16 +8949,16 @@
         <v>1.0</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>140</v>
+        <v>156</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>13</v>
@@ -8754,16 +8970,16 @@
         <v>1.0</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>142</v>
+        <v>158</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>144</v>
+        <v>160</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>13</v>
@@ -8775,16 +8991,16 @@
         <v>2.0</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>145</v>
+        <v>161</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>146</v>
+        <v>162</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>13</v>
@@ -8796,16 +9012,16 @@
         <v>2.0</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>13</v>
@@ -8817,16 +9033,16 @@
         <v>2.0</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>148</v>
+        <v>164</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>13</v>
@@ -8838,16 +9054,16 @@
         <v>2.0</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>148</v>
+        <v>164</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>150</v>
+        <v>166</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>13</v>
@@ -8859,16 +9075,16 @@
         <v>2.0</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>151</v>
+        <v>167</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F17" s="8" t="s">
         <v>13</v>
@@ -8880,16 +9096,16 @@
         <v>3.0</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>153</v>
+        <v>169</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>13</v>
@@ -8901,16 +9117,16 @@
         <v>3.0</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>13</v>
@@ -8922,16 +9138,16 @@
         <v>3.0</v>
       </c>
       <c r="B20" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="D20" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="C20" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>139</v>
-      </c>
       <c r="E20" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>13</v>
@@ -8946,13 +9162,13 @@
         <v>45669.0</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F21" s="8" t="s">
         <v>13</v>
@@ -8967,13 +9183,13 @@
         <v>45659.0</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F22" s="8" t="s">
         <v>13</v>
@@ -8988,13 +9204,13 @@
         <v>45669.0</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F23" s="8" t="s">
         <v>13</v>
@@ -9009,13 +9225,13 @@
         <v>45728.0</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F24" s="8" t="s">
         <v>13</v>
@@ -9030,13 +9246,13 @@
         <v>45728.0</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F25" s="8" t="s">
         <v>13</v>
@@ -9051,13 +9267,13 @@
         <v>45728.0</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="D26" s="8" t="s">
         <v>23</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F26" s="8" t="s">
         <v>13</v>
@@ -9072,13 +9288,13 @@
         <v>45728.0</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F27" s="8" t="s">
         <v>13</v>
@@ -9093,13 +9309,13 @@
         <v>45728.0</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F28" s="8" t="s">
         <v>13</v>
@@ -9114,13 +9330,13 @@
         <v>45789.0</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F29" s="8" t="s">
         <v>13</v>
@@ -9135,13 +9351,13 @@
         <v>45789.0</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F30" s="8" t="s">
         <v>13</v>
@@ -9156,13 +9372,13 @@
         <v>45789.0</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F31" s="8" t="s">
         <v>13</v>
@@ -9177,13 +9393,13 @@
         <v>45881.0</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F32" s="8" t="s">
         <v>13</v>
@@ -9198,13 +9414,13 @@
         <v>45881.0</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F33" s="8" t="s">
         <v>13</v>
@@ -9219,13 +9435,13 @@
         <v>45881.0</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F34" s="8" t="s">
         <v>13</v>
@@ -9240,13 +9456,13 @@
         <v>45942.0</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F35" s="8" t="s">
         <v>13</v>
@@ -9261,13 +9477,13 @@
         <v>45942.0</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F36" s="8" t="s">
         <v>13</v>
@@ -9282,13 +9498,13 @@
         <v>45942.0</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F37" s="8" t="s">
         <v>13</v>
@@ -9303,13 +9519,13 @@
         <v>45942.0</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F38" s="8" t="s">
         <v>13</v>
@@ -9324,13 +9540,13 @@
         <v>45973.0</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F39" s="8" t="s">
         <v>13</v>
@@ -9345,13 +9561,13 @@
         <v>46003.0</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F40" s="8" t="s">
         <v>13</v>
@@ -9366,13 +9582,13 @@
         <v>46003.0</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F41" s="8" t="s">
         <v>13</v>
@@ -9384,16 +9600,16 @@
         <v>5.0</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F42" s="8" t="s">
         <v>13</v>
@@ -9567,7 +9783,7 @@
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
       <c r="D61" s="3" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
@@ -10566,7 +10782,7 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>171</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4" ht="29.25" customHeight="1"/>
@@ -10606,40 +10822,40 @@
       <c r="A7" s="21">
         <v>1.0</v>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="13">
         <v>45941.0</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>172</v>
+        <v>188</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="F7" s="21" t="s">
         <v>13</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="17">
         <v>1.0</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="13">
         <v>45941.0</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>13</v>
@@ -10651,16 +10867,16 @@
         <v>1.0</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>177</v>
+        <v>193</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="F9" s="17" t="s">
         <v>13</v>
@@ -10672,22 +10888,22 @@
         <v>1.0</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>178</v>
+        <v>194</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="F10" s="17" t="s">
         <v>13</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>179</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -10695,16 +10911,16 @@
         <v>2.0</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>180</v>
+        <v>196</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>181</v>
+        <v>197</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="F11" s="17" t="s">
         <v>13</v>
@@ -10716,23 +10932,23 @@
         <v>2.0</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>13</v>
       </c>
       <c r="G12" s="21"/>
       <c r="I12" s="22" t="s">
-        <v>183</v>
+        <v>199</v>
       </c>
     </row>
     <row r="13">
@@ -10740,22 +10956,22 @@
         <v>2.0</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>184</v>
+        <v>200</v>
       </c>
       <c r="D13" s="17" t="s">
         <v>23</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="F13" s="17" t="s">
         <v>13</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>185</v>
+        <v>201</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
@@ -10763,16 +10979,16 @@
         <v>2.0</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>186</v>
+        <v>202</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="F14" s="17" t="s">
         <v>13</v>
@@ -10784,16 +11000,16 @@
         <v>2.0</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>187</v>
+        <v>203</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="F15" s="17" t="s">
         <v>13</v>
@@ -10805,16 +11021,16 @@
         <v>3.0</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>188</v>
+        <v>204</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="F16" s="17" t="s">
         <v>13</v>
@@ -10826,16 +11042,16 @@
         <v>3.0</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>189</v>
+        <v>205</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="F17" s="17" t="s">
         <v>13</v>
@@ -10847,39 +11063,39 @@
         <v>3.0</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>191</v>
+        <v>207</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="F18" s="17" t="s">
         <v>13</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>192</v>
+        <v>208</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="17">
         <v>4.0</v>
       </c>
-      <c r="B19" s="12">
+      <c r="B19" s="13">
         <v>45669.0</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>193</v>
+        <v>209</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="F19" s="17" t="s">
         <v>13</v>
@@ -10890,17 +11106,17 @@
       <c r="A20" s="17">
         <v>4.0</v>
       </c>
-      <c r="B20" s="12">
+      <c r="B20" s="13">
         <v>45700.0</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>194</v>
+        <v>210</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="F20" s="17" t="s">
         <v>13</v>
@@ -10911,17 +11127,17 @@
       <c r="A21" s="17">
         <v>4.0</v>
       </c>
-      <c r="B21" s="12">
+      <c r="B21" s="13">
         <v>45728.0</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>195</v>
+        <v>211</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>196</v>
+        <v>212</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="F21" s="17" t="s">
         <v>13</v>
@@ -10932,17 +11148,17 @@
       <c r="A22" s="17">
         <v>4.0</v>
       </c>
-      <c r="B22" s="12">
+      <c r="B22" s="13">
         <v>45728.0</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>197</v>
+        <v>213</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="F22" s="17" t="s">
         <v>13</v>
@@ -10953,17 +11169,17 @@
       <c r="A23" s="17">
         <v>4.0</v>
       </c>
-      <c r="B23" s="12">
+      <c r="B23" s="13">
         <v>45759.0</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>198</v>
+        <v>214</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>199</v>
+        <v>215</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="F23" s="17" t="s">
         <v>13</v>
@@ -10974,17 +11190,17 @@
       <c r="A24" s="17">
         <v>4.0</v>
       </c>
-      <c r="B24" s="12">
+      <c r="B24" s="13">
         <v>45789.0</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>200</v>
+        <v>216</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="F24" s="17" t="s">
         <v>13</v>
@@ -10995,17 +11211,17 @@
       <c r="A25" s="17">
         <v>4.0</v>
       </c>
-      <c r="B25" s="12">
+      <c r="B25" s="13">
         <v>45820.0</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>198</v>
+        <v>214</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="F25" s="17" t="s">
         <v>13</v>
@@ -11016,17 +11232,17 @@
       <c r="A26" s="17">
         <v>5.0</v>
       </c>
-      <c r="B26" s="12">
+      <c r="B26" s="13">
         <v>45881.0</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="F26" s="17" t="s">
         <v>13</v>
@@ -11037,17 +11253,17 @@
       <c r="A27" s="17">
         <v>5.0</v>
       </c>
-      <c r="B27" s="12">
+      <c r="B27" s="13">
         <v>45942.0</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>202</v>
+        <v>218</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="F27" s="17" t="s">
         <v>13</v>
@@ -11058,17 +11274,17 @@
       <c r="A28" s="17">
         <v>5.0</v>
       </c>
-      <c r="B28" s="12">
+      <c r="B28" s="13">
         <v>45942.0</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>203</v>
+        <v>219</v>
       </c>
       <c r="D28" s="8" t="s">
         <v>23</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="F28" s="17" t="s">
         <v>13</v>
@@ -11079,17 +11295,17 @@
       <c r="A29" s="17">
         <v>5.0</v>
       </c>
-      <c r="B29" s="12">
+      <c r="B29" s="13">
         <v>46003.0</v>
       </c>
       <c r="C29" s="17" t="s">
-        <v>204</v>
+        <v>220</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="F29" s="17" t="s">
         <v>13</v>
@@ -11100,17 +11316,17 @@
       <c r="A30" s="17">
         <v>5.0</v>
       </c>
-      <c r="B30" s="12">
+      <c r="B30" s="13">
         <v>46003.0</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>205</v>
+        <v>221</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="F30" s="17" t="s">
         <v>13</v>
@@ -11122,16 +11338,16 @@
         <v>5.0</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="F31" s="17" t="s">
         <v>13</v>
@@ -11314,7 +11530,7 @@
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
       <c r="D51" s="3" t="s">
-        <v>207</v>
+        <v>223</v>
       </c>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
@@ -12319,10 +12535,10 @@
         <v>0</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>208</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>130</v>
+        <v>224</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>146</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
@@ -12330,7 +12546,7 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>209</v>
+        <v>225</v>
       </c>
     </row>
     <row r="4" ht="29.25" customHeight="1"/>
@@ -12397,19 +12613,19 @@
         <v>45971.0</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>210</v>
+        <v>226</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>211</v>
+        <v>227</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
@@ -12420,13 +12636,13 @@
         <v>45974.0</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>212</v>
+        <v>228</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>13</v>
@@ -12441,19 +12657,19 @@
         <v>45978.0</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>214</v>
+        <v>230</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>215</v>
+        <v>231</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -12464,13 +12680,13 @@
         <v>45973.0</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>216</v>
+        <v>232</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>13</v>
@@ -12485,13 +12701,13 @@
         <v>45973.0</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>218</v>
+        <v>234</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>13</v>
@@ -12506,13 +12722,13 @@
         <v>45971.0</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>220</v>
+        <v>236</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>13</v>
@@ -12527,13 +12743,13 @@
         <v>45973.0</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>13</v>
@@ -12548,13 +12764,13 @@
         <v>45973.0</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>222</v>
+        <v>238</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>13</v>
@@ -12569,13 +12785,13 @@
         <v>45973.0</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>223</v>
+        <v>239</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>13</v>
@@ -12590,19 +12806,19 @@
         <v>45978.0</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>224</v>
+        <v>240</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>225</v>
+        <v>241</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F17" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>226</v>
+        <v>242</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
@@ -12613,13 +12829,13 @@
         <v>45979.0</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>227</v>
+        <v>243</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>13</v>
@@ -12634,13 +12850,13 @@
         <v>45980.0</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>228</v>
+        <v>244</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>13</v>
@@ -12655,13 +12871,13 @@
         <v>45981.0</v>
       </c>
       <c r="C20" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="E20" s="8" t="s">
         <v>229</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>230</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>213</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>13</v>
@@ -12676,13 +12892,13 @@
         <v>45981.0</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>231</v>
+        <v>247</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>232</v>
+        <v>248</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F21" s="8" t="s">
         <v>13</v>
@@ -12697,19 +12913,19 @@
         <v>45985.0</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>233</v>
+        <v>249</v>
       </c>
       <c r="D22" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F22" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>234</v>
+        <v>250</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -12720,13 +12936,13 @@
         <v>45987.0</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>235</v>
+        <v>251</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F23" s="8" t="s">
         <v>13</v>
@@ -12741,13 +12957,13 @@
         <v>45988.0</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>236</v>
+        <v>252</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>230</v>
+        <v>246</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F24" s="8" t="s">
         <v>13</v>
@@ -12762,19 +12978,19 @@
         <v>45988.0</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>237</v>
+        <v>253</v>
       </c>
       <c r="D25" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F25" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>238</v>
+        <v>254</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
@@ -12785,13 +13001,13 @@
         <v>45989.0</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>239</v>
+        <v>255</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F26" s="8" t="s">
         <v>13</v>
@@ -12806,13 +13022,13 @@
         <v>45992.0</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>240</v>
+        <v>256</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>241</v>
+        <v>257</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F27" s="8" t="s">
         <v>13</v>
@@ -12827,13 +13043,13 @@
         <v>45992.0</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>242</v>
+        <v>258</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>243</v>
+        <v>259</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>244</v>
+        <v>260</v>
       </c>
       <c r="F28" s="8" t="s">
         <v>13</v>
@@ -12848,19 +13064,19 @@
         <v>45992.0</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>245</v>
+        <v>261</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="F29" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>246</v>
+        <v>262</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
@@ -12871,13 +13087,13 @@
         <v>45992.0</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F30" s="8" t="s">
         <v>13</v>
@@ -12892,13 +13108,13 @@
         <v>45992.0</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>248</v>
+        <v>264</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>244</v>
+        <v>260</v>
       </c>
       <c r="F31" s="8" t="s">
         <v>13</v>
@@ -12913,13 +13129,13 @@
         <v>45994.0</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>249</v>
+        <v>265</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>232</v>
+        <v>248</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F32" s="8" t="s">
         <v>13</v>
@@ -12934,13 +13150,13 @@
         <v>45994.0</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>250</v>
+        <v>266</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F33" s="8" t="s">
         <v>13</v>
@@ -12955,13 +13171,13 @@
         <v>45997.0</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>251</v>
+        <v>267</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>252</v>
+        <v>268</v>
       </c>
       <c r="F34" s="8" t="s">
         <v>13</v>
@@ -12976,13 +13192,13 @@
         <v>45999.0</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>253</v>
+        <v>269</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F35" s="8" t="s">
         <v>13</v>
@@ -12997,13 +13213,13 @@
         <v>45999.0</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>254</v>
+        <v>270</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>225</v>
+        <v>241</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>255</v>
+        <v>271</v>
       </c>
       <c r="F36" s="8" t="s">
         <v>13</v>
@@ -13018,13 +13234,13 @@
         <v>46001.0</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>256</v>
+        <v>272</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F37" s="8" t="s">
         <v>13</v>
@@ -13039,13 +13255,13 @@
         <v>46001.0</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>257</v>
+        <v>273</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F38" s="8" t="s">
         <v>13</v>
@@ -13060,13 +13276,13 @@
         <v>46003.0</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>258</v>
+        <v>274</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>255</v>
+        <v>271</v>
       </c>
       <c r="F39" s="8" t="s">
         <v>13</v>
@@ -13078,16 +13294,16 @@
         <v>5.0</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>259</v>
+        <v>275</v>
       </c>
       <c r="D40" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="F40" s="8" t="s">
         <v>13</v>
@@ -13189,7 +13405,7 @@
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
       <c r="D51" s="3" t="s">
-        <v>260</v>
+        <v>276</v>
       </c>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
@@ -14188,7 +14404,7 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>261</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" ht="29.25" customHeight="1"/>
@@ -14225,22 +14441,22 @@
       </c>
     </row>
     <row r="7" ht="16.5" customHeight="1">
-      <c r="A7" s="11">
+      <c r="A7" s="12">
         <v>1.0</v>
       </c>
       <c r="B7" s="24">
         <v>45971.0</v>
       </c>
-      <c r="C7" s="11" t="s">
-        <v>262</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>255</v>
-      </c>
-      <c r="F7" s="11" t="s">
+      <c r="C7" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="F7" s="12" t="s">
         <v>13</v>
       </c>
       <c r="G7" s="6"/>
@@ -14253,13 +14469,13 @@
         <v>46002.0</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>263</v>
+        <v>279</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>23</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>13</v>
@@ -14271,20 +14487,20 @@
         <v>1.0</v>
       </c>
       <c r="B9" s="25" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="C9" s="25" t="s">
-        <v>265</v>
+        <v>281</v>
       </c>
       <c r="D9" s="25" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E9" s="25" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
       <c r="F9" s="26"/>
       <c r="G9" s="25" t="s">
-        <v>266</v>
+        <v>282</v>
       </c>
     </row>
     <row r="10" ht="33.0" customHeight="1">
@@ -14292,16 +14508,16 @@
         <v>1.0</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>142</v>
+        <v>158</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>267</v>
+        <v>283</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>23</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>13</v>
@@ -14313,16 +14529,16 @@
         <v>2.0</v>
       </c>
       <c r="B11" s="25" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>268</v>
+        <v>284</v>
       </c>
       <c r="D11" s="25" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="E11" s="25" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
       <c r="F11" s="25" t="s">
         <v>13</v>
@@ -14334,16 +14550,16 @@
         <v>2.0</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>269</v>
+        <v>285</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>270</v>
+        <v>286</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>255</v>
+        <v>271</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>13</v>
@@ -14355,16 +14571,16 @@
         <v>2.0</v>
       </c>
       <c r="B13" s="25" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>271</v>
+        <v>287</v>
       </c>
       <c r="D13" s="25" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="E13" s="25" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
       <c r="F13" s="25" t="s">
         <v>13</v>
@@ -14376,16 +14592,16 @@
         <v>2.0</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>272</v>
+        <v>288</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>13</v>
@@ -14397,16 +14613,16 @@
         <v>2.0</v>
       </c>
       <c r="B15" s="25" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>273</v>
+        <v>289</v>
       </c>
       <c r="D15" s="25" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E15" s="25" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
       <c r="F15" s="25" t="s">
         <v>13</v>
@@ -14418,16 +14634,16 @@
         <v>2.0</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>274</v>
+        <v>290</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>23</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>255</v>
+        <v>271</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>13</v>
@@ -14439,16 +14655,16 @@
         <v>3.0</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>275</v>
+        <v>291</v>
       </c>
       <c r="D17" s="25" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E17" s="25" t="s">
-        <v>255</v>
+        <v>271</v>
       </c>
       <c r="F17" s="25" t="s">
         <v>13</v>
@@ -14460,16 +14676,16 @@
         <v>3.0</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>276</v>
+        <v>292</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>270</v>
+        <v>286</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>13</v>
@@ -14481,16 +14697,16 @@
         <v>3.0</v>
       </c>
       <c r="B19" s="25" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>277</v>
+        <v>293</v>
       </c>
       <c r="D19" s="25" t="s">
-        <v>270</v>
+        <v>286</v>
       </c>
       <c r="E19" s="25" t="s">
-        <v>255</v>
+        <v>271</v>
       </c>
       <c r="F19" s="25" t="s">
         <v>13</v>
@@ -14502,16 +14718,16 @@
         <v>3.0</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>278</v>
+        <v>294</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>279</v>
+        <v>295</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>13</v>
@@ -14526,13 +14742,13 @@
         <v>45669.0</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>277</v>
+        <v>293</v>
       </c>
       <c r="D21" s="25" t="s">
-        <v>270</v>
+        <v>286</v>
       </c>
       <c r="E21" s="25" t="s">
-        <v>255</v>
+        <v>271</v>
       </c>
       <c r="F21" s="25" t="s">
         <v>13</v>
@@ -14543,17 +14759,17 @@
       <c r="A22" s="8">
         <v>4.0</v>
       </c>
-      <c r="B22" s="13">
+      <c r="B22" s="10">
         <v>45700.0</v>
       </c>
       <c r="C22" s="8" t="s">
+        <v>296</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="E22" s="8" t="s">
         <v>280</v>
-      </c>
-      <c r="D22" s="8" t="s">
-        <v>281</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>264</v>
       </c>
       <c r="F22" s="8" t="s">
         <v>13</v>
@@ -14568,13 +14784,13 @@
         <v>45728.0</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>277</v>
+        <v>293</v>
       </c>
       <c r="D23" s="25" t="s">
         <v>23</v>
       </c>
       <c r="E23" s="25" t="s">
-        <v>255</v>
+        <v>271</v>
       </c>
       <c r="F23" s="25" t="s">
         <v>13</v>
@@ -14585,17 +14801,17 @@
       <c r="A24" s="8">
         <v>4.0</v>
       </c>
-      <c r="B24" s="13">
+      <c r="B24" s="10">
         <v>45759.0</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>282</v>
+        <v>298</v>
       </c>
       <c r="D24" s="8" t="s">
         <v>23</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
       <c r="F24" s="8" t="s">
         <v>13</v>
@@ -14610,13 +14826,13 @@
         <v>45850.0</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>283</v>
+        <v>299</v>
       </c>
       <c r="D25" s="25" t="s">
         <v>23</v>
       </c>
       <c r="E25" s="25" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
       <c r="F25" s="25" t="s">
         <v>13</v>
@@ -14627,17 +14843,17 @@
       <c r="A26" s="8">
         <v>5.0</v>
       </c>
-      <c r="B26" s="13">
+      <c r="B26" s="10">
         <v>45881.0</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>200</v>
+        <v>216</v>
       </c>
       <c r="D26" s="8" t="s">
         <v>23</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>255</v>
+        <v>271</v>
       </c>
       <c r="F26" s="8" t="s">
         <v>13</v>
@@ -14652,13 +14868,13 @@
         <v>45942.0</v>
       </c>
       <c r="C27" s="25" t="s">
-        <v>284</v>
+        <v>300</v>
       </c>
       <c r="D27" s="25" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E27" s="25" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
       <c r="F27" s="25" t="s">
         <v>13</v>
@@ -14673,13 +14889,13 @@
         <v>46003.0</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>285</v>
+        <v>301</v>
       </c>
       <c r="D28" s="8" t="s">
         <v>23</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>255</v>
+        <v>271</v>
       </c>
       <c r="F28" s="8" t="s">
         <v>13</v>
@@ -14691,16 +14907,16 @@
         <v>5.0</v>
       </c>
       <c r="B29" s="25" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
       <c r="C29" s="25" t="s">
+        <v>302</v>
+      </c>
+      <c r="D29" s="25" t="s">
         <v>286</v>
       </c>
-      <c r="D29" s="25" t="s">
-        <v>270</v>
-      </c>
       <c r="E29" s="25" t="s">
-        <v>264</v>
+        <v>280</v>
       </c>
       <c r="F29" s="25" t="s">
         <v>13</v>
@@ -14883,7 +15099,7 @@
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
       <c r="D49" s="3" t="s">
-        <v>287</v>
+        <v>303</v>
       </c>
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>

</xml_diff>